<commit_message>
Fix four practice-test defects: incomplete PDF extraction, D36 unpriced lines, BOQ-content detectors, defaulted region/currency
- project_index: 'Extracted - incomplete' when a Quantity header and units have no numbers in the text layer
- D36 lists every unpriced/unmapped BOQ line; exceptions no longer headed 'resolved'
- detectors scan all imported text columns, extra markers, near-duplicate sizes
- migration 0016 projects.basis_defaulted; confirm_basis/action; banner, completeness, readiness gate
- 6 regression tests; 3 fixtures now pass region/currency explicitly; practice test re-run; full suite 464 passed

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ShGswK3SJJeEsEzfdZjprk
</commit_message>
<xml_diff>
--- a/practice_test/real_document/generated/PRJ-9201_tender_pack_r1/PRJ-9201-D10_r1_Commercial-clarifications.xlsx
+++ b/practice_test/real_document/generated/PRJ-9201_tender_pack_r1/PRJ-9201-D10_r1_Commercial-clarifications.xlsx
@@ -682,7 +682,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>TQ-PRJ-9201-027</t>
+          <t>TQ-PRJ-9201-031</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -713,7 +713,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>TQ-PRJ-9201-028</t>
+          <t>TQ-PRJ-9201-032</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -744,7 +744,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>TQ-PRJ-9201-029</t>
+          <t>TQ-PRJ-9201-033</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -775,7 +775,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>TQ-PRJ-9201-036</t>
+          <t>TQ-PRJ-9201-040</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">

</xml_diff>